<commit_message>
Updated metadata generator, mainly associated with agents
</commit_message>
<xml_diff>
--- a/sources/xlsx/Agents.xlsx
+++ b/sources/xlsx/Agents.xlsx
@@ -3,16 +3,17 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9060" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="7710" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="meta" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="agents" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="map" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="RDF-Relations" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="relations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="map" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="RDF-Relations" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -21,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -84,13 +85,21 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Consolas"/>
-      <color rgb="001F4E79"/>
+      <color rgb="FF1F4E79"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -102,17 +111,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBF3FB"/>
+        <fgColor rgb="FFEBF3FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -126,26 +135,26 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -157,9 +166,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -169,9 +176,14 @@
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -593,9 +605,9 @@
   <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="16.44140625" customWidth="1" style="14" min="1" max="1"/>
-    <col width="19.109375" customWidth="1" style="14" min="2" max="2"/>
-    <col width="121.109375" bestFit="1" customWidth="1" style="14" min="3" max="3"/>
+    <col width="16.44140625" customWidth="1" style="15" min="1" max="1"/>
+    <col width="19.109375" customWidth="1" style="15" min="2" max="2"/>
+    <col width="121.109375" bestFit="1" customWidth="1" style="15" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -606,128 +618,128 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Created</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="3" t="n">
         <v>20260512</v>
       </c>
-      <c r="C3" s="6" t="n"/>
+      <c r="C3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Modified</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="3" t="n">
         <v>20260512</v>
       </c>
-      <c r="C4" s="6" t="n"/>
+      <c r="C4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Submitted</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="3" t="n">
         <v>20260512</v>
       </c>
-      <c r="C5" s="6" t="n"/>
+      <c r="C5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Ongoing*</t>
         </is>
       </c>
-      <c r="C6" s="12" t="n"/>
+      <c r="C6" s="17" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Primary Contact</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="8" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Contact Name</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Ben Norton</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n"/>
+      <c r="C9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Organization</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Yale University</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n"/>
+      <c r="C10" s="9" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>ben.norton@yale.edu</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n"/>
+      <c r="C11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="12" t="n"/>
+      <c r="A12" s="17" t="n"/>
+      <c r="B12" s="17" t="n"/>
+      <c r="C12" s="17" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Concept Scheme Annotation Properties</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/1LFrSqBu77SraEJN6zpjMvn6MF8rIcOnQIMt-_8LxTA4/edit?gid=1334808172#gid=1334808172</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Concept Annotation Properties</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/1LFrSqBu77SraEJN6zpjMvn6MF8rIcOnQIMt-_8LxTA4/edit?gid=1986942826#gid=1986942826</t>
         </is>
@@ -762,122 +774,128 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.2"/>
   <cols>
-    <col width="40" customWidth="1" style="12" min="1" max="1"/>
-    <col width="28" customWidth="1" style="12" min="2" max="3"/>
-    <col width="22" customWidth="1" style="12" min="4" max="4"/>
-    <col width="36" bestFit="1" customWidth="1" style="12" min="5" max="5"/>
-    <col width="18.88671875" bestFit="1" customWidth="1" style="12" min="6" max="6"/>
-    <col width="41.77734375" customWidth="1" style="12" min="7" max="7"/>
-    <col width="42.6640625" customWidth="1" style="12" min="8" max="8"/>
-    <col width="8.33203125" bestFit="1" customWidth="1" style="12" min="9" max="9"/>
-    <col width="37.5546875" bestFit="1" customWidth="1" style="12" min="10" max="10"/>
-    <col width="32" customWidth="1" style="12" min="11" max="11"/>
-    <col width="22" customWidth="1" style="12" min="12" max="12"/>
-    <col width="36.21875" bestFit="1" customWidth="1" style="12" min="13" max="13"/>
-    <col width="30" customWidth="1" style="12" min="14" max="14"/>
-    <col width="113" bestFit="1" customWidth="1" style="12" min="15" max="15"/>
-    <col width="8.88671875" customWidth="1" style="12" min="16" max="16384"/>
+    <col width="40" customWidth="1" style="17" min="1" max="1"/>
+    <col width="28" customWidth="1" style="17" min="2" max="3"/>
+    <col width="22" customWidth="1" style="17" min="4" max="4"/>
+    <col width="36" bestFit="1" customWidth="1" style="17" min="5" max="5"/>
+    <col width="18.88671875" bestFit="1" customWidth="1" style="17" min="6" max="6"/>
+    <col width="32.5546875" customWidth="1" style="17" min="7" max="7"/>
+    <col width="29" customWidth="1" style="17" min="8" max="8"/>
+    <col width="8.33203125" bestFit="1" customWidth="1" style="17" min="9" max="9"/>
+    <col width="37.5546875" bestFit="1" customWidth="1" style="17" min="10" max="10"/>
+    <col width="32" customWidth="1" style="17" min="11" max="11"/>
+    <col width="22" customWidth="1" style="17" min="12" max="12"/>
+    <col width="36.21875" bestFit="1" customWidth="1" style="17" min="13" max="13"/>
+    <col width="30" customWidth="1" style="17" min="14" max="14"/>
+    <col width="113" bestFit="1" customWidth="1" style="17" min="15" max="15"/>
+    <col width="8.88671875" customWidth="1" style="17" min="16" max="16"/>
+    <col width="8.88671875" customWidth="1" style="17" min="17" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>agentURI</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>blankNodeLabel</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>agentName</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>agentType</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="17" t="inlineStr">
         <is>
           <t>orcidURI</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="17" t="inlineStr">
         <is>
           <t>agentEmail</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="17" t="inlineStr">
         <is>
           <t>agentURL</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="17" t="inlineStr">
         <is>
           <t>agentHomepage</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="17" t="inlineStr">
         <is>
           <t>acronym</t>
         </is>
       </c>
-      <c r="J1" s="12" t="inlineStr">
+      <c r="J1" s="17" t="inlineStr">
         <is>
           <t>memberOfURI</t>
         </is>
       </c>
-      <c r="K1" s="12" t="inlineStr">
+      <c r="K1" s="17" t="inlineStr">
         <is>
           <t>memberOfName</t>
         </is>
       </c>
-      <c r="L1" s="12" t="inlineStr">
+      <c r="L1" s="17" t="inlineStr">
         <is>
           <t>memberOfRole</t>
         </is>
       </c>
-      <c r="M1" s="12" t="inlineStr">
+      <c r="M1" s="17" t="inlineStr">
         <is>
           <t>parentOrgURI</t>
         </is>
       </c>
-      <c r="N1" s="12" t="inlineStr">
+      <c r="N1" s="17" t="inlineStr">
         <is>
           <t>parentOrgName</t>
         </is>
       </c>
-      <c r="O1" s="12" t="inlineStr">
+      <c r="O1" s="17" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1" s="14">
-      <c r="A2" s="12" t="inlineStr">
+    <row r="2" ht="18" customHeight="1" s="15">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>https://kos.geospecimens.org/org/ben-norton</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>agent_ben_norton</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
         <is>
           <t>Ben Norton</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="D2" s="17" t="inlineStr">
         <is>
           <t>schema:Person</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="E2" s="17" t="inlineStr">
         <is>
           <t>https://orcid.org/0000-0002-5819-9134</t>
         </is>
       </c>
-      <c r="F2" s="12" t="inlineStr">
+      <c r="F2" s="17" t="inlineStr">
         <is>
           <t>ben.norton@yale.edu</t>
         </is>
@@ -887,153 +905,153 @@
           <t>https://mbnorton.com</t>
         </is>
       </c>
-      <c r="J2" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="K2" s="12" t="inlineStr">
+      <c r="J2" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="K2" s="17" t="inlineStr">
         <is>
           <t>Mineralogy Extension Task Group</t>
         </is>
       </c>
-      <c r="L2" s="12" t="inlineStr">
+      <c r="L2" s="17" t="inlineStr">
         <is>
           <t>co-convener</t>
         </is>
       </c>
-      <c r="M2" s="12" t="inlineStr">
+      <c r="M2" s="17" t="inlineStr">
         <is>
           <t>https://kos.geospecimens.org/org/yale-university</t>
         </is>
       </c>
-      <c r="N2" s="12" t="inlineStr">
+      <c r="N2" s="17" t="inlineStr">
         <is>
           <t>Yale University</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1" s="14">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
+    <row r="3" ht="18" customHeight="1" s="15">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>agent_mineralogy_extension_task_group</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>Mineralogy Extension Task Group</t>
         </is>
       </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>schema:Organization</t>
         </is>
       </c>
-      <c r="G3" s="12" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>https://www.tdwg.org/community/esp/mineralogy/</t>
         </is>
       </c>
-      <c r="H3" s="12" t="inlineStr">
+      <c r="H3" s="17" t="inlineStr">
         <is>
           <t>https://www.tdwg.org/community/esp/mineralogy/</t>
         </is>
       </c>
-      <c r="I3" s="12" t="inlineStr">
+      <c r="I3" s="17" t="inlineStr">
         <is>
           <t>MinExt</t>
         </is>
       </c>
-      <c r="J3" s="12" t="inlineStr">
+      <c r="J3" s="17" t="inlineStr">
         <is>
           <t>https://kos.geospecimens.org/org/tdwg</t>
         </is>
       </c>
-      <c r="K3" s="12" t="inlineStr">
+      <c r="K3" s="17" t="inlineStr">
         <is>
           <t>Biodiversity Information Standards</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1" s="14">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="4" ht="18" customHeight="1" s="15">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>https://kos.geospecimens.org/org/tdwg</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>agent_biodiversity_information_standards</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>Biodiversity Information Standards</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>schema:Organization</t>
         </is>
       </c>
-      <c r="G4" s="12" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr">
         <is>
           <t>https://www.tdwg.org</t>
         </is>
       </c>
-      <c r="H4" s="12" t="inlineStr">
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>https://www.tdwg.org</t>
         </is>
       </c>
-      <c r="I4" s="12" t="inlineStr">
+      <c r="I4" s="17" t="inlineStr">
         <is>
           <t>TDWG</t>
         </is>
       </c>
-      <c r="O4" s="12" t="inlineStr">
+      <c r="O4" s="17" t="inlineStr">
         <is>
           <t>Taxonomic Databases Working Group, now Biodiversity Information Standards</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1" s="14">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="5" ht="18" customHeight="1" s="15">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>https://kos.geospecimens.org/org/yale-university</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>agent_yale_university</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>Yale University</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>schema:Organization</t>
         </is>
       </c>
-      <c r="G5" s="12" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>https://www.yale.edu</t>
         </is>
       </c>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>https://www.yale.edu</t>
         </is>
       </c>
-      <c r="O5" s="12" t="inlineStr">
+      <c r="O5" s="17" t="inlineStr">
         <is>
           <t>Also identified by GBIF GRSciColl IRI: https://scientific-collections.gbif.org/institution/75f50140-830d-4630-a290-3d6e951a7c29</t>
         </is>
@@ -1056,371 +1074,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="45.109375" customWidth="1" style="14" min="1" max="1"/>
-    <col width="61.109375" customWidth="1" style="14" min="2" max="2"/>
+    <col width="37.33203125" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
+    <col width="40.109375" bestFit="1" customWidth="1" style="15" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="14.4" customHeight="1" s="15">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>agentURI</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>resourceURI</t>
-        </is>
-      </c>
-      <c r="C1" s="12" t="inlineStr">
-        <is>
-          <t>hadRole</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>relatedAgentURI</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>agentRole</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.4" customHeight="1" s="15">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>https://kos.geospecimens.org/org/ben-norton</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/hazard-type</t>
-        </is>
-      </c>
-      <c r="C2" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:publisher</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/yale-university</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/standards/elementset/agrelon#hasEmployer</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="14.4" customHeight="1" s="15">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/tdwg</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>https://www.w3.org/ns/org#unitOf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="14.4" customHeight="1" s="15">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>https://kos.geospecimens.org/org/ben-norton</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/hazard-type</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:author</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/hazard-type</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:editor</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/hazard-type</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:custodian</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/ben-norton</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/aggregate-form</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:publisher</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/ben-norton</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/aggregate-form</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:author</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/aggregate-form</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:editor</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/aggregate-form</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:custodian</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/ben-norton</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/constituent-part-proportion</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:publisher</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/ben-norton</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/constituent-part-proportion</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:author</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/constituent-part-proportion</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:editor</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/constituent-part-proportion</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:custodian</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/ben-norton</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/geological-specimen-material-type</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:publisher</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/ben-norton</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/geological-specimen-material-type</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:author</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/geological-specimen-material-type</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:editor</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/geological-specimen-material-type</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:custodian</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/ben-norton</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/geological-specimen-name-type</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:publisher</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/ben-norton</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/geological-specimen-name-type</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:author</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/geological-specimen-name-type</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:editor</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>https://kos.resources.org/def/geological-specimen-name-type</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>isoroles:custodian</t>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/standards/elementset/agrelon#isMemberOf</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1431,200 +1168,617 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="54" customWidth="1" style="14" min="1" max="1"/>
-    <col width="54" customWidth="1" style="14" min="2" max="2"/>
-    <col width="44" customWidth="1" style="14" min="3" max="3"/>
+    <col width="45.109375" customWidth="1" style="15" min="1" max="1"/>
+    <col width="61.109375" customWidth="1" style="15" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" s="14">
-      <c r="A1" s="15" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>agentURI</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>resourceURI</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>hadRole</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="16" customHeight="1" s="14">
-      <c r="A2" s="16" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>https://kos.geospecimens.org/org/ben-norton</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/hazard-type</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:publisher</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/ben-norton</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/hazard-type</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:author</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/hazard-type</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/hazard-type</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:custodian</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/ben-norton</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>https://kos.resources.org/def/aggregate-form</t>
         </is>
       </c>
-      <c r="C2" s="16" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:publisher</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/ben-norton</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/aggregate-form</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:author</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/aggregate-form</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/aggregate-form</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:custodian</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/ben-norton</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/constituent-part-proportion</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:publisher</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/ben-norton</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/constituent-part-proportion</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:author</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/constituent-part-proportion</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/constituent-part-proportion</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:custodian</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/ben-norton</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/geological-specimen-material-type</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:publisher</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/ben-norton</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/geological-specimen-material-type</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:author</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/geological-specimen-material-type</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/geological-specimen-material-type</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:custodian</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/ben-norton</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/geological-specimen-name-type</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:publisher</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/ben-norton</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/geological-specimen-name-type</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:author</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/geological-specimen-name-type</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/geological-specimen-name-type</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>isoroles:custodian</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="54" customWidth="1" style="15" min="1" max="2"/>
+    <col width="44" customWidth="1" style="15" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="19.95" customHeight="1" s="15">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>agentURI</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>resourceURI</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>hadRole</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16.05" customHeight="1" s="15">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/ben-norton</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>https://kos.resources.org/def/aggregate-form</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>isoroles:editor, isoroles:publisher</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="16" customHeight="1" s="14">
-      <c r="A3" s="17" t="inlineStr">
+    <row r="3" ht="16.05" customHeight="1" s="15">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>https://kos.geospecimens.org/org/ben-norton</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>https://kos.resources.org/def/constituent-part-proportion</t>
         </is>
       </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>isoroles:editor, isoroles:publisher</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="16" customHeight="1" s="14">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="4" ht="16.05" customHeight="1" s="15">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>https://kos.geospecimens.org/org/ben-norton</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>https://kos.resources.org/def/geological-specimen-material-type</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>isoroles:editor, isoroles:publisher</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="16" customHeight="1" s="14">
-      <c r="A5" s="17" t="inlineStr">
+    <row r="5" ht="16.05" customHeight="1" s="15">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>https://kos.geospecimens.org/org/ben-norton</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>https://kos.resources.org/def/geological-specimen-name-type</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>isoroles:editor, isoroles:publisher</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="16" customHeight="1" s="14">
-      <c r="A6" s="16" t="inlineStr">
+    <row r="6" ht="16.05" customHeight="1" s="15">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>https://kos.geospecimens.org/org/ben-norton</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>https://kos.resources.org/def/hazard-type</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>isoroles:editor, isoroles:publisher</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="16" customHeight="1" s="14">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
+    <row r="7" ht="16.05" customHeight="1" s="15">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>https://kos.resources.org/def/aggregate-form</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>isoroles:contributor, isoroles:custodian</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="16" customHeight="1" s="14">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
+    <row r="8" ht="16.05" customHeight="1" s="15">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>https://kos.resources.org/def/constituent-part-proportion</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>isoroles:contributor, isoroles:custodian</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="16" customHeight="1" s="14">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B9" s="17" t="inlineStr">
+    <row r="9" ht="16.05" customHeight="1" s="15">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>https://kos.resources.org/def/geological-specimen-material-type</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>isoroles:contributor, isoroles:custodian</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1" s="14">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B10" s="16" t="inlineStr">
+    <row r="10" ht="16.05" customHeight="1" s="15">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>https://kos.resources.org/def/geological-specimen-name-type</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>isoroles:contributor, isoroles:custodian</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1" s="14">
-      <c r="A11" s="17" t="inlineStr">
-        <is>
-          <t>https://kos.geospecimens.org/org/minext</t>
-        </is>
-      </c>
-      <c r="B11" s="17" t="inlineStr">
+    <row r="11" ht="16.05" customHeight="1" s="15">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>https://kos.geospecimens.org/org/minext</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>https://kos.resources.org/def/hazard-type</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr">
         <is>
           <t>isoroles:contributor, isoroles:custodian</t>
         </is>
       </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>https://www.w3.org/ns/org#unitOf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>https://www.w3.org/ns/org#memberOf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>https://www.w3.org/ns/org#hasMember</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/standards/elementset/agrelon#hasEmployer</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>